<commit_message>
Adapt to the regtest tool exports and the SharePoint timeline
- Timeline: import the SharePoint list export directly (group rows, environments,
  OT version, substitutes for absences, duplicates), data-quality tab, plan the
  next release by shifting a whole release, export back in the list layout
- Errors & runs: Error Management import with per-import change history
  (new, status changed, more runs, gone) and the regtest window
- Test cases & coverage: catalogue from the list or tree export, RegTest
  documents from Document Management in the coverage matrix
- Admin > Pages: hide pages and rename menu entries; PO sessions hidden by default
- Header row detection skips title rows; fictional sample exports and demo data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJfoB5ttuydBGveMAN9LwA
</commit_message>
<xml_diff>
--- a/sample-data/bugs_export.xlsx
+++ b/sample-data/bugs_export.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>R-2026.4</t>
+          <t>V8.3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>R-2026.4</t>
+          <t>V8.3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>